<commit_message>
trainign stride equal to 4 for testing 1
</commit_message>
<xml_diff>
--- a/Excel Results/results_explicit.xlsx
+++ b/Excel Results/results_explicit.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -474,6 +474,11 @@
           <t>explicit_feature_4</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>explicit_feature_5</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -501,6 +506,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -528,6 +538,11 @@
           <t>explicit_feature</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>explicit_feature</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -555,6 +570,11 @@
           <t>img_local_context_ROI_1</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>img_local_context_ROI_1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -582,6 +602,11 @@
           <t>None</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -609,6 +634,11 @@
           <t>None</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -636,6 +666,11 @@
           <t>None</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -663,6 +698,11 @@
           <t>1</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -690,6 +730,11 @@
           <t>400</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -713,6 +758,11 @@
         </is>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -728,6 +778,7 @@
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -739,6 +790,7 @@
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -750,6 +802,7 @@
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -777,6 +830,11 @@
           <t>27432</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>27432</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -800,6 +858,11 @@
         </is>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>7011</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>7011</t>
         </is>
@@ -815,6 +878,7 @@
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -842,6 +906,11 @@
           <t>7011</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>7011</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -869,6 +938,11 @@
           <t>True</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -896,6 +970,11 @@
           <t>None</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -923,6 +1002,11 @@
           <t>Embedding_Temporal_LSTM</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Embedding_Temporal_LSTM</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -946,6 +1030,11 @@
         </is>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -961,6 +1050,7 @@
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -988,6 +1078,11 @@
           <t>head</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1015,6 +1110,11 @@
           <t>LSTM</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1042,6 +1142,11 @@
           <t>112</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1069,6 +1174,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1096,6 +1206,11 @@
           <t>1</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1123,6 +1238,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1150,6 +1270,11 @@
           <t>112</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1177,6 +1302,11 @@
           <t>0.25</t>
         </is>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1200,6 +1330,11 @@
         </is>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>128</t>
         </is>
@@ -1215,6 +1350,7 @@
       <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1242,6 +1378,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1265,6 +1406,11 @@
         </is>
       </c>
       <c r="E34" t="inlineStr">
+        <is>
+          <t>literature_classes</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
         <is>
           <t>literature_classes</t>
         </is>
@@ -1280,6 +1426,7 @@
       <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1291,6 +1438,7 @@
       <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1318,6 +1466,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1345,6 +1498,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1372,6 +1530,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1399,6 +1562,11 @@
           <t>0.0001</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>0.0001</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1426,6 +1594,11 @@
           <t>1e-05</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1e-05</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1453,6 +1626,11 @@
           <t>Adam</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1480,6 +1658,11 @@
           <t>0.0009</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>0.0009</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1507,6 +1690,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1534,6 +1722,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1561,6 +1754,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1588,6 +1786,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1615,6 +1818,11 @@
           <t>0.1</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1642,6 +1850,11 @@
           <t>0.9</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1669,6 +1882,11 @@
           <t>0</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1696,6 +1914,11 @@
           <t>FocalLoss</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>FocalLoss</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1723,6 +1946,11 @@
           <t>1</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1750,6 +1978,11 @@
           <t>explicit_feature_4</t>
         </is>
       </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>explicit_feature_5</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1777,6 +2010,11 @@
           <t>None</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1800,6 +2038,11 @@
         </is>
       </c>
       <c r="E55" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -1815,6 +2058,7 @@
       <c r="C56" s="2" t="inlineStr"/>
       <c r="D56" s="2" t="inlineStr"/>
       <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1826,6 +2070,7 @@
       <c r="C57" s="2" t="inlineStr"/>
       <c r="D57" s="2" t="inlineStr"/>
       <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1837,6 +2082,7 @@
       <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="2" t="inlineStr"/>
       <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1848,6 +2094,7 @@
       <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="2" t="inlineStr"/>
       <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1859,6 +2106,7 @@
       <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="2" t="inlineStr"/>
       <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1870,6 +2118,7 @@
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="2" t="inlineStr"/>
       <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1897,6 +2146,11 @@
           <t>0.841</t>
         </is>
       </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>0.843</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1924,6 +2178,11 @@
           <t>0.884</t>
         </is>
       </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>0.884</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1951,6 +2210,11 @@
           <t>0.885</t>
         </is>
       </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>0.885</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1978,6 +2242,11 @@
           <t>0.884</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>0.884</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2005,6 +2274,11 @@
           <t>0.882</t>
         </is>
       </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>0.883</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2032,6 +2306,11 @@
           <t>0.86</t>
         </is>
       </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>0.858</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2059,6 +2338,11 @@
           <t>0.827</t>
         </is>
       </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>0.832</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2086,6 +2370,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2109,6 +2398,11 @@
         </is>
       </c>
       <c r="E70" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
         <is>
           <t>9</t>
         </is>
@@ -2124,6 +2418,7 @@
       <c r="C71" s="2" t="inlineStr"/>
       <c r="D71" s="2" t="inlineStr"/>
       <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2151,6 +2446,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2178,6 +2478,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2205,6 +2510,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2228,6 +2538,11 @@
         </is>
       </c>
       <c r="E75" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2243,6 +2558,7 @@
       <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="2" t="inlineStr"/>
       <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="B77" s="2" t="inlineStr">
@@ -2265,6 +2581,11 @@
           <t>False</t>
         </is>
       </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="2" t="inlineStr">
@@ -2287,6 +2608,11 @@
           <t>./output/dataset_cache</t>
         </is>
       </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>./output/dataset_cache</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="2" t="inlineStr">
@@ -2309,6 +2635,11 @@
           <t>0.5</t>
         </is>
       </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="2" t="inlineStr">
@@ -2331,6 +2662,11 @@
           <t>0.7</t>
         </is>
       </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="2" t="inlineStr">
@@ -2353,6 +2689,11 @@
           <t>True</t>
         </is>
       </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="B82" s="2" t="inlineStr">
@@ -2375,6 +2716,11 @@
           <t>True</t>
         </is>
       </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="B83" s="2" t="inlineStr">
@@ -2397,6 +2743,11 @@
           <t>10</t>
         </is>
       </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="B84" s="2" t="inlineStr">
@@ -2417,6 +2768,18 @@
       <c r="E84" t="inlineStr">
         <is>
           <t>5</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
         </is>
       </c>
     </row>

</xml_diff>